<commit_message>
Improved deprecation / breaking changes notice with compatibility info
</commit_message>
<xml_diff>
--- a/Java_Deprecation_Report.xlsx
+++ b/Java_Deprecation_Report.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="192">
   <si>
     <t>Type</t>
   </si>
@@ -603,6 +603,12 @@
   </si>
   <si>
     <t>deprecatedProperty</t>
+  </si>
+  <si>
+    <t>7.0</t>
+  </si>
+  <si>
+    <t>2026-09-13</t>
   </si>
   <si>
     <t>MyPojoRequest</t>
@@ -3772,36 +3778,36 @@
         <v>11</v>
       </c>
       <c r="G102" t="s" s="11">
-        <v>11</v>
+        <v>188</v>
       </c>
       <c r="H102" t="s" s="11">
-        <v>11</v>
+        <v>189</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="9">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B103" t="s" s="9">
         <v>186</v>
       </c>
       <c r="C103" t="s" s="9">
+        <v>191</v>
+      </c>
+      <c r="D103" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="E103" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F103" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G103" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H103" t="s" s="11">
         <v>189</v>
-      </c>
-      <c r="D103" t="s" s="9">
-        <v>11</v>
-      </c>
-      <c r="E103" t="s" s="9">
-        <v>11</v>
-      </c>
-      <c r="F103" t="s" s="10">
-        <v>11</v>
-      </c>
-      <c r="G103" t="s" s="11">
-        <v>11</v>
-      </c>
-      <c r="H103" t="s" s="11">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented and tested handling of deprecated parameters
</commit_message>
<xml_diff>
--- a/Java_Deprecation_Report.xlsx
+++ b/Java_Deprecation_Report.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="193">
   <si>
     <t>Type</t>
   </si>
@@ -615,6 +615,9 @@
   </si>
   <si>
     <t>formerMandatoryRequestProperty</t>
+  </si>
+  <si>
+    <t>MyContext</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1124,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E1136C3-A1B3-DD42-A00A-DCFCD8D149EA}">
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="9" width="31.5"/>
@@ -3810,6 +3813,32 @@
         <v>189</v>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="s" s="9">
+        <v>192</v>
+      </c>
+      <c r="B104" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C104" t="s" s="9">
+        <v>63</v>
+      </c>
+      <c r="D104" t="s" s="9">
+        <v>63</v>
+      </c>
+      <c r="E104" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F104" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G104" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H104" t="s" s="11">
+        <v>189</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Validation groups for constraints (#744)
</commit_message>
<xml_diff>
--- a/Java_Deprecation_Report.xlsx
+++ b/Java_Deprecation_Report.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="193">
   <si>
     <t>Type</t>
   </si>
@@ -605,10 +605,19 @@
     <t>deprecatedProperty</t>
   </si>
   <si>
+    <t>7.0</t>
+  </si>
+  <si>
+    <t>2026-09-13</t>
+  </si>
+  <si>
     <t>MyPojoRequest</t>
   </si>
   <si>
     <t>formerMandatoryRequestProperty</t>
+  </si>
+  <si>
+    <t>MyContext</t>
   </si>
 </sst>
 </file>
@@ -1115,7 +1124,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E1136C3-A1B3-DD42-A00A-DCFCD8D149EA}">
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="9" width="31.5"/>
@@ -3772,36 +3781,62 @@
         <v>11</v>
       </c>
       <c r="G102" t="s" s="11">
-        <v>11</v>
+        <v>188</v>
       </c>
       <c r="H102" t="s" s="11">
-        <v>11</v>
+        <v>189</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="9">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B103" t="s" s="9">
         <v>186</v>
       </c>
       <c r="C103" t="s" s="9">
+        <v>191</v>
+      </c>
+      <c r="D103" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="E103" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F103" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G103" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H103" t="s" s="11">
         <v>189</v>
       </c>
-      <c r="D103" t="s" s="9">
-        <v>11</v>
-      </c>
-      <c r="E103" t="s" s="9">
-        <v>11</v>
-      </c>
-      <c r="F103" t="s" s="10">
-        <v>11</v>
-      </c>
-      <c r="G103" t="s" s="11">
-        <v>11</v>
-      </c>
-      <c r="H103" t="s" s="11">
-        <v>11</v>
+    </row>
+    <row r="104">
+      <c r="A104" t="s" s="9">
+        <v>192</v>
+      </c>
+      <c r="B104" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C104" t="s" s="9">
+        <v>63</v>
+      </c>
+      <c r="D104" t="s" s="9">
+        <v>63</v>
+      </c>
+      <c r="E104" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F104" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G104" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H104" t="s" s="11">
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prepared development of next version
</commit_message>
<xml_diff>
--- a/Java_Deprecation_Report.xlsx
+++ b/Java_Deprecation_Report.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="203">
   <si>
     <t>Type</t>
   </si>
@@ -617,7 +617,37 @@
     <t>formerMandatoryRequestProperty</t>
   </si>
   <si>
+    <t>MultiVersioningTestService</t>
+  </si>
+  <si>
+    <t>deprecatedEndpoint</t>
+  </si>
+  <si>
+    <t>I'm so deprecated.</t>
+  </si>
+  <si>
     <t>MyContext</t>
+  </si>
+  <si>
+    <t>ClientType</t>
+  </si>
+  <si>
+    <t>CLIENT_3</t>
+  </si>
+  <si>
+    <t>DeprecatedClass</t>
+  </si>
+  <si>
+    <t>DeprecatedOpenAPIDataType</t>
+  </si>
+  <si>
+    <t>AnotherDeprecatedRESTService</t>
+  </si>
+  <si>
+    <t>operationOfADeprecatedService</t>
+  </si>
+  <si>
+    <t>DeprecatedOpenAPIEnum</t>
   </si>
 </sst>
 </file>
@@ -1124,7 +1154,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E1136C3-A1B3-DD42-A00A-DCFCD8D149EA}">
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="9" width="31.5"/>
@@ -3821,13 +3851,13 @@
         <v>186</v>
       </c>
       <c r="C104" t="s" s="9">
-        <v>63</v>
+        <v>193</v>
       </c>
       <c r="D104" t="s" s="9">
-        <v>63</v>
+        <v>11</v>
       </c>
       <c r="E104" t="s" s="9">
-        <v>11</v>
+        <v>194</v>
       </c>
       <c r="F104" t="s" s="10">
         <v>11</v>
@@ -3836,6 +3866,188 @@
         <v>188</v>
       </c>
       <c r="H104" t="s" s="11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s" s="9">
+        <v>195</v>
+      </c>
+      <c r="B105" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C105" t="s" s="9">
+        <v>63</v>
+      </c>
+      <c r="D105" t="s" s="9">
+        <v>63</v>
+      </c>
+      <c r="E105" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F105" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G105" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H105" t="s" s="11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s" s="9">
+        <v>196</v>
+      </c>
+      <c r="B106" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C106" t="s" s="9">
+        <v>197</v>
+      </c>
+      <c r="D106" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="E106" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F106" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G106" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H106" t="s" s="11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s" s="9">
+        <v>198</v>
+      </c>
+      <c r="B107" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C107" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="D107" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="E107" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F107" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G107" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H107" t="s" s="11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s" s="9">
+        <v>199</v>
+      </c>
+      <c r="B108" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C108" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="D108" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="E108" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F108" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G108" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H108" t="s" s="11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s" s="9">
+        <v>200</v>
+      </c>
+      <c r="B109" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C109" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="D109" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="E109" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F109" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G109" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H109" t="s" s="11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s" s="9">
+        <v>200</v>
+      </c>
+      <c r="B110" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C110" t="s" s="9">
+        <v>201</v>
+      </c>
+      <c r="D110" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="E110" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F110" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G110" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H110" t="s" s="11">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s" s="9">
+        <v>202</v>
+      </c>
+      <c r="B111" t="s" s="9">
+        <v>186</v>
+      </c>
+      <c r="C111" t="s" s="9">
+        <v>202</v>
+      </c>
+      <c r="D111" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="E111" t="s" s="9">
+        <v>11</v>
+      </c>
+      <c r="F111" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="G111" t="s" s="11">
+        <v>188</v>
+      </c>
+      <c r="H111" t="s" s="11">
         <v>189</v>
       </c>
     </row>

</xml_diff>